<commit_message>
feat: automate Shioaji pricing and backfill ETF holdings
</commit_message>
<xml_diff>
--- a/archive/2026-04/ETF_Investment_Portfolio_20260407.xlsx
+++ b/archive/2026-04/ETF_Investment_Portfolio_20260407.xlsx
@@ -454,559 +454,559 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2330</t>
+          <t>2059</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>台積電</t>
+          <t>川湖</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>806000</v>
+        <v>191000</v>
       </c>
       <c r="D2" t="n">
-        <v>7.0208</v>
+        <v>3.0747</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2383</t>
+          <t>2308</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>台光電</t>
+          <t>台達電</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>323000</v>
+        <v>280000</v>
       </c>
       <c r="D3" t="n">
-        <v>4.3291</v>
+        <v>1.9269</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2345</t>
+          <t>2330</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>智邦</t>
+          <t>台積電</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>531000</v>
+        <v>806000</v>
       </c>
       <c r="D4" t="n">
-        <v>4.0632</v>
+        <v>7.0208</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3017</t>
+          <t>2337</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>奇鋐</t>
+          <t>旺宏</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>370000</v>
+        <v>671000</v>
       </c>
       <c r="D5" t="n">
-        <v>3.6859</v>
+        <v>0.4165</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6223</t>
+          <t>2344</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>旺矽</t>
+          <t>華邦電</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>196000</v>
+        <v>663000</v>
       </c>
       <c r="D6" t="n">
-        <v>3.5513</v>
+        <v>0.2929</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6515</t>
+          <t>2345</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>智邦</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>111000</v>
+        <v>531000</v>
       </c>
       <c r="D7" t="n">
-        <v>3.5283</v>
+        <v>4.0632</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3533</t>
+          <t>2360</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>嘉澤</t>
+          <t>致茂</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>343000</v>
+        <v>370000</v>
       </c>
       <c r="D8" t="n">
-        <v>3.3757</v>
+        <v>2.7333</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8299</t>
+          <t>2368</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>群聯</t>
+          <t>金像電</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>434000</v>
+        <v>227000</v>
       </c>
       <c r="D9" t="n">
-        <v>3.2478</v>
+        <v>0.9886</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3037</t>
+          <t>2383</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>台光電</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1277000</v>
+        <v>323000</v>
       </c>
       <c r="D10" t="n">
-        <v>3.1896</v>
+        <v>4.3291</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3105</t>
+          <t>2408</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>穩懋</t>
+          <t>南亞科</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1716000</v>
+        <v>2432000</v>
       </c>
       <c r="D11" t="n">
-        <v>3.1051</v>
+        <v>2.3466</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3163</t>
+          <t>2449</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>波若威</t>
+          <t>京元電子</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>676000</v>
+        <v>166000</v>
       </c>
       <c r="D12" t="n">
-        <v>3.0971</v>
+        <v>0.2069</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2059</t>
+          <t>2486</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>川湖</t>
+          <t>一詮</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>191000</v>
+        <v>1230000</v>
       </c>
       <c r="D13" t="n">
-        <v>3.0747</v>
+        <v>0.882</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>6442</t>
+          <t>3017</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>奇鋐</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>310000</v>
+        <v>370000</v>
       </c>
       <c r="D14" t="n">
-        <v>2.9838</v>
+        <v>3.6859</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8996</t>
+          <t>3036</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>高力</t>
+          <t>文曄</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>715000</v>
+        <v>947000</v>
       </c>
       <c r="D15" t="n">
-        <v>2.9799</v>
+        <v>1.0208</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2360</t>
+          <t>3037</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>致茂</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>370000</v>
+        <v>1277000</v>
       </c>
       <c r="D16" t="n">
-        <v>2.7333</v>
+        <v>3.1896</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>7769</t>
+          <t>3081</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>鴻勁</t>
+          <t>聯亞</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>142000</v>
+        <v>185000</v>
       </c>
       <c r="D17" t="n">
-        <v>2.6207</v>
+        <v>1.6248</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6669</t>
+          <t>3105</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>緯穎</t>
+          <t>穩懋</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>146000</v>
+        <v>1716000</v>
       </c>
       <c r="D18" t="n">
-        <v>2.3959</v>
+        <v>3.1051</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2408</t>
+          <t>3131</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>南亞科</t>
+          <t>弘塑</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2432000</v>
+        <v>87000</v>
       </c>
       <c r="D19" t="n">
-        <v>2.3466</v>
+        <v>1.2937</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>8046</t>
+          <t>3163</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>南電</t>
+          <t>波若威</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>858000</v>
+        <v>676000</v>
       </c>
       <c r="D20" t="n">
-        <v>2.3453</v>
+        <v>3.0971</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>7751</t>
+          <t>3189</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>竑騰</t>
+          <t>景碩</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>285000</v>
+        <v>457013</v>
       </c>
       <c r="D21" t="n">
-        <v>2.2836</v>
+        <v>0.739</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6510</t>
+          <t>3260</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>精測</t>
+          <t>威剛</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>142000</v>
+        <v>231000</v>
       </c>
       <c r="D22" t="n">
-        <v>2.1629</v>
+        <v>0.4018</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4749</t>
+          <t>3324</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>新應材</t>
+          <t>雙鴻</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>526000</v>
+        <v>93000</v>
       </c>
       <c r="D23" t="n">
-        <v>2.0276</v>
+        <v>0.4072</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>6805</t>
+          <t>3443</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>富世達</t>
+          <t>創意</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>219000</v>
+        <v>66000</v>
       </c>
       <c r="D24" t="n">
-        <v>1.9867</v>
+        <v>0.7369</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2308</t>
+          <t>3491</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>台達電</t>
+          <t>昇達科</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>280000</v>
+        <v>71000</v>
       </c>
       <c r="D25" t="n">
-        <v>1.9269</v>
+        <v>0.5108</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>8358</t>
+          <t>3529</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>金居</t>
+          <t>力旺</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1728000</v>
+        <v>67000</v>
       </c>
       <c r="D26" t="n">
-        <v>1.9127</v>
+        <v>0.848</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3653</t>
+          <t>3533</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>健策</t>
+          <t>嘉澤</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>100000</v>
+        <v>343000</v>
       </c>
       <c r="D27" t="n">
-        <v>1.7854</v>
+        <v>3.3757</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5274</t>
+          <t>3653</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>信驊</t>
+          <t>健策</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>29000</v>
+        <v>100000</v>
       </c>
       <c r="D28" t="n">
-        <v>1.6315</v>
+        <v>1.7854</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>3081</t>
+          <t>3661</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>聯亞</t>
+          <t>世芯-KY</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>185000</v>
+        <v>59000</v>
       </c>
       <c r="D29" t="n">
-        <v>1.6248</v>
+        <v>0.768</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6584</t>
+          <t>3665</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>南俊國際</t>
+          <t>貿聯-KY</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>566000</v>
+        <v>100000</v>
       </c>
       <c r="D30" t="n">
-        <v>1.5526</v>
+        <v>0.9216</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3131</t>
+          <t>3711</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>弘塑</t>
+          <t>日月光投控</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>87000</v>
+        <v>236000</v>
       </c>
       <c r="D31" t="n">
-        <v>1.2937</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5347</t>
+          <t>4749</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>世界</t>
+          <t>新應材</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2277000</v>
+        <v>526000</v>
       </c>
       <c r="D32" t="n">
-        <v>1.2054</v>
+        <v>2.0276</v>
       </c>
     </row>
     <row r="33">
@@ -1030,361 +1030,361 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>3036</t>
+          <t>5274</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>文曄</t>
+          <t>信驊</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>947000</v>
+        <v>29000</v>
       </c>
       <c r="D34" t="n">
-        <v>1.0208</v>
+        <v>1.6315</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2368</t>
+          <t>5289</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>金像電</t>
+          <t>宜鼎</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>227000</v>
+        <v>90000</v>
       </c>
       <c r="D35" t="n">
-        <v>0.9886</v>
+        <v>0.4145</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>3665</t>
+          <t>5347</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>貿聯-KY</t>
+          <t>世界</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>100000</v>
+        <v>2277000</v>
       </c>
       <c r="D36" t="n">
-        <v>0.9216</v>
+        <v>1.2054</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>6781</t>
+          <t>6223</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>AES-KY</t>
+          <t>旺矽</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>198000</v>
+        <v>196000</v>
       </c>
       <c r="D37" t="n">
-        <v>0.9119</v>
+        <v>3.5513</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2486</t>
+          <t>6274</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>一詮</t>
+          <t>台燿</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1230000</v>
+        <v>230000</v>
       </c>
       <c r="D38" t="n">
-        <v>0.882</v>
+        <v>0.6873</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3529</t>
+          <t>6442</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>力旺</t>
+          <t>光聖</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>67000</v>
+        <v>310000</v>
       </c>
       <c r="D39" t="n">
-        <v>0.848</v>
+        <v>2.9838</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>6531</t>
+          <t>6510</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>愛普*</t>
+          <t>精測</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>367000</v>
+        <v>142000</v>
       </c>
       <c r="D40" t="n">
-        <v>0.7771</v>
+        <v>2.1629</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>3661</t>
+          <t>6515</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>世芯-KY</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>59000</v>
+        <v>111000</v>
       </c>
       <c r="D41" t="n">
-        <v>0.768</v>
+        <v>3.5283</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>3189</t>
+          <t>6531</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>457013</v>
+        <v>367000</v>
       </c>
       <c r="D42" t="n">
-        <v>0.739</v>
+        <v>0.7771</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>3443</t>
+          <t>6584</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>創意</t>
+          <t>南俊國際</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>66000</v>
+        <v>566000</v>
       </c>
       <c r="D43" t="n">
-        <v>0.7369</v>
+        <v>1.5526</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>6274</t>
+          <t>6669</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>台燿</t>
+          <t>緯穎</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>230000</v>
+        <v>146000</v>
       </c>
       <c r="D44" t="n">
-        <v>0.6873</v>
+        <v>2.3959</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>8021</t>
+          <t>6781</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>尖點</t>
+          <t>AES-KY</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>569920</v>
+        <v>198000</v>
       </c>
       <c r="D45" t="n">
-        <v>0.6651</v>
+        <v>0.9119</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>3491</t>
+          <t>6805</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>昇達科</t>
+          <t>富世達</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>71000</v>
+        <v>219000</v>
       </c>
       <c r="D46" t="n">
-        <v>0.5108</v>
+        <v>1.9867</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2337</t>
+          <t>7751</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>旺宏</t>
+          <t>竑騰</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>671000</v>
+        <v>285000</v>
       </c>
       <c r="D47" t="n">
-        <v>0.4165</v>
+        <v>2.2836</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>5289</t>
+          <t>7769</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>宜鼎</t>
+          <t>鴻勁</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>90000</v>
+        <v>142000</v>
       </c>
       <c r="D48" t="n">
-        <v>0.4145</v>
+        <v>2.6207</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>3711</t>
+          <t>8021</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>日月光投控</t>
+          <t>尖點</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>236000</v>
+        <v>569920</v>
       </c>
       <c r="D49" t="n">
-        <v>0.41</v>
+        <v>0.6651</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>3324</t>
+          <t>8046</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>雙鴻</t>
+          <t>南電</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>93000</v>
+        <v>858000</v>
       </c>
       <c r="D50" t="n">
-        <v>0.4072</v>
+        <v>2.3453</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>3260</t>
+          <t>8299</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>威剛</t>
+          <t>群聯</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>231000</v>
+        <v>434000</v>
       </c>
       <c r="D51" t="n">
-        <v>0.4018</v>
+        <v>3.2478</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2344</t>
+          <t>8358</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>華邦電</t>
+          <t>金居</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>663000</v>
+        <v>1728000</v>
       </c>
       <c r="D52" t="n">
-        <v>0.2929</v>
+        <v>1.9127</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2449</t>
+          <t>8996</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>京元電子</t>
+          <t>高力</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>166000</v>
+        <v>715000</v>
       </c>
       <c r="D53" t="n">
-        <v>0.2069</v>
+        <v>2.9799</v>
       </c>
     </row>
   </sheetData>
@@ -1431,589 +1431,589 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2330</t>
+          <t>2059</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>台積電</t>
+          <t>川湖</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>806000</v>
+        <v>191000</v>
       </c>
       <c r="D2" t="n">
-        <v>7.0208</v>
+        <v>3.0747</v>
       </c>
       <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2383</t>
+          <t>2308</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>台光電</t>
+          <t>台達電</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>323000</v>
+        <v>280000</v>
       </c>
       <c r="D3" t="n">
-        <v>4.3291</v>
+        <v>1.9269</v>
       </c>
       <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2345</t>
+          <t>2330</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>智邦</t>
+          <t>台積電</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>531000</v>
+        <v>806000</v>
       </c>
       <c r="D4" t="n">
-        <v>4.0632</v>
+        <v>7.0208</v>
       </c>
       <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3017</t>
+          <t>2337</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>奇鋐</t>
+          <t>旺宏</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>370000</v>
+        <v>671000</v>
       </c>
       <c r="D5" t="n">
-        <v>3.6859</v>
+        <v>0.4165</v>
       </c>
       <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6223</t>
+          <t>2344</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>旺矽</t>
+          <t>華邦電</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>196000</v>
+        <v>663000</v>
       </c>
       <c r="D6" t="n">
-        <v>3.5513</v>
+        <v>0.2929</v>
       </c>
       <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6515</t>
+          <t>2345</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>智邦</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>111000</v>
+        <v>531000</v>
       </c>
       <c r="D7" t="n">
-        <v>3.5283</v>
+        <v>4.0632</v>
       </c>
       <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3533</t>
+          <t>2360</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>嘉澤</t>
+          <t>致茂</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>343000</v>
+        <v>370000</v>
       </c>
       <c r="D8" t="n">
-        <v>3.3757</v>
+        <v>2.7333</v>
       </c>
       <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8299</t>
+          <t>2368</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>群聯</t>
+          <t>金像電</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>434000</v>
+        <v>227000</v>
       </c>
       <c r="D9" t="n">
-        <v>3.2478</v>
+        <v>0.9886</v>
       </c>
       <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3037</t>
+          <t>2383</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>台光電</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1277000</v>
+        <v>323000</v>
       </c>
       <c r="D10" t="n">
-        <v>3.1896</v>
+        <v>4.3291</v>
       </c>
       <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3105</t>
+          <t>2408</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>穩懋</t>
+          <t>南亞科</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1716000</v>
+        <v>2432000</v>
       </c>
       <c r="D11" t="n">
-        <v>3.1051</v>
+        <v>2.3466</v>
       </c>
       <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3163</t>
+          <t>2449</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>波若威</t>
+          <t>京元電子</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>676000</v>
+        <v>166000</v>
       </c>
       <c r="D12" t="n">
-        <v>3.0971</v>
+        <v>0.2069</v>
       </c>
       <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2059</t>
+          <t>2486</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>川湖</t>
+          <t>一詮</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>191000</v>
+        <v>1230000</v>
       </c>
       <c r="D13" t="n">
-        <v>3.0747</v>
+        <v>0.882</v>
       </c>
       <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>6442</t>
+          <t>3017</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>奇鋐</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>310000</v>
+        <v>370000</v>
       </c>
       <c r="D14" t="n">
-        <v>2.9838</v>
+        <v>3.6859</v>
       </c>
       <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8996</t>
+          <t>3036</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>高力</t>
+          <t>文曄</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>715000</v>
+        <v>947000</v>
       </c>
       <c r="D15" t="n">
-        <v>2.9799</v>
+        <v>1.0208</v>
       </c>
       <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2360</t>
+          <t>3037</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>致茂</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>370000</v>
+        <v>1277000</v>
       </c>
       <c r="D16" t="n">
-        <v>2.7333</v>
+        <v>3.1896</v>
       </c>
       <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>7769</t>
+          <t>3081</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>鴻勁</t>
+          <t>聯亞</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>142000</v>
+        <v>185000</v>
       </c>
       <c r="D17" t="n">
-        <v>2.6207</v>
+        <v>1.6248</v>
       </c>
       <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6669</t>
+          <t>3105</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>緯穎</t>
+          <t>穩懋</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>146000</v>
+        <v>1716000</v>
       </c>
       <c r="D18" t="n">
-        <v>2.3959</v>
+        <v>3.1051</v>
       </c>
       <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2408</t>
+          <t>3131</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>南亞科</t>
+          <t>弘塑</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2432000</v>
+        <v>87000</v>
       </c>
       <c r="D19" t="n">
-        <v>2.3466</v>
+        <v>1.2937</v>
       </c>
       <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>8046</t>
+          <t>3163</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>南電</t>
+          <t>波若威</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>858000</v>
+        <v>676000</v>
       </c>
       <c r="D20" t="n">
-        <v>2.3453</v>
+        <v>3.0971</v>
       </c>
       <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>7751</t>
+          <t>3189</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>竑騰</t>
+          <t>景碩</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>285000</v>
+        <v>457013</v>
       </c>
       <c r="D21" t="n">
-        <v>2.2836</v>
+        <v>0.739</v>
       </c>
       <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6510</t>
+          <t>3260</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>精測</t>
+          <t>威剛</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>142000</v>
+        <v>231000</v>
       </c>
       <c r="D22" t="n">
-        <v>2.1629</v>
+        <v>0.4018</v>
       </c>
       <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4749</t>
+          <t>3324</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>新應材</t>
+          <t>雙鴻</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>526000</v>
+        <v>93000</v>
       </c>
       <c r="D23" t="n">
-        <v>2.0276</v>
+        <v>0.4072</v>
       </c>
       <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>6805</t>
+          <t>3443</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>富世達</t>
+          <t>創意</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>219000</v>
+        <v>66000</v>
       </c>
       <c r="D24" t="n">
-        <v>1.9867</v>
+        <v>0.7369</v>
       </c>
       <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2308</t>
+          <t>3491</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>台達電</t>
+          <t>昇達科</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>280000</v>
+        <v>71000</v>
       </c>
       <c r="D25" t="n">
-        <v>1.9269</v>
+        <v>0.5108</v>
       </c>
       <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>8358</t>
+          <t>3529</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>金居</t>
+          <t>力旺</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1728000</v>
+        <v>67000</v>
       </c>
       <c r="D26" t="n">
-        <v>1.9127</v>
+        <v>0.848</v>
       </c>
       <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3653</t>
+          <t>3533</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>健策</t>
+          <t>嘉澤</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>100000</v>
+        <v>343000</v>
       </c>
       <c r="D27" t="n">
-        <v>1.7854</v>
+        <v>3.3757</v>
       </c>
       <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5274</t>
+          <t>3653</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>信驊</t>
+          <t>健策</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>29000</v>
+        <v>100000</v>
       </c>
       <c r="D28" t="n">
-        <v>1.6315</v>
+        <v>1.7854</v>
       </c>
       <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>3081</t>
+          <t>3661</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>聯亞</t>
+          <t>世芯-KY</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>185000</v>
+        <v>59000</v>
       </c>
       <c r="D29" t="n">
-        <v>1.6248</v>
+        <v>0.768</v>
       </c>
       <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6584</t>
+          <t>3665</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>南俊國際</t>
+          <t>貿聯-KY</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>566000</v>
+        <v>100000</v>
       </c>
       <c r="D30" t="n">
-        <v>1.5526</v>
+        <v>0.9216</v>
       </c>
       <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3131</t>
+          <t>3711</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>弘塑</t>
+          <t>日月光投控</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>87000</v>
+        <v>236000</v>
       </c>
       <c r="D31" t="n">
-        <v>1.2937</v>
+        <v>0.41</v>
       </c>
       <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5347</t>
+          <t>4749</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>世界</t>
+          <t>新應材</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2277000</v>
+        <v>526000</v>
       </c>
       <c r="D32" t="n">
-        <v>1.2054</v>
+        <v>2.0276</v>
       </c>
       <c r="E32" t="inlineStr"/>
     </row>
@@ -2039,380 +2039,380 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>3036</t>
+          <t>5274</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>文曄</t>
+          <t>信驊</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>947000</v>
+        <v>29000</v>
       </c>
       <c r="D34" t="n">
-        <v>1.0208</v>
+        <v>1.6315</v>
       </c>
       <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2368</t>
+          <t>5289</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>金像電</t>
+          <t>宜鼎</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>227000</v>
+        <v>90000</v>
       </c>
       <c r="D35" t="n">
-        <v>0.9886</v>
+        <v>0.4145</v>
       </c>
       <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>3665</t>
+          <t>5347</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>貿聯-KY</t>
+          <t>世界</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>100000</v>
+        <v>2277000</v>
       </c>
       <c r="D36" t="n">
-        <v>0.9216</v>
+        <v>1.2054</v>
       </c>
       <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>6781</t>
+          <t>6223</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>AES-KY</t>
+          <t>旺矽</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>198000</v>
+        <v>196000</v>
       </c>
       <c r="D37" t="n">
-        <v>0.9119</v>
+        <v>3.5513</v>
       </c>
       <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2486</t>
+          <t>6274</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>一詮</t>
+          <t>台燿</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1230000</v>
+        <v>230000</v>
       </c>
       <c r="D38" t="n">
-        <v>0.882</v>
+        <v>0.6873</v>
       </c>
       <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3529</t>
+          <t>6442</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>力旺</t>
+          <t>光聖</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>67000</v>
+        <v>310000</v>
       </c>
       <c r="D39" t="n">
-        <v>0.848</v>
+        <v>2.9838</v>
       </c>
       <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>6531</t>
+          <t>6510</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>愛普*</t>
+          <t>精測</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>367000</v>
+        <v>142000</v>
       </c>
       <c r="D40" t="n">
-        <v>0.7771</v>
+        <v>2.1629</v>
       </c>
       <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>3661</t>
+          <t>6515</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>世芯-KY</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>59000</v>
+        <v>111000</v>
       </c>
       <c r="D41" t="n">
-        <v>0.768</v>
+        <v>3.5283</v>
       </c>
       <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>3189</t>
+          <t>6531</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>457013</v>
+        <v>367000</v>
       </c>
       <c r="D42" t="n">
-        <v>0.739</v>
+        <v>0.7771</v>
       </c>
       <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>3443</t>
+          <t>6584</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>創意</t>
+          <t>南俊國際</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>66000</v>
+        <v>566000</v>
       </c>
       <c r="D43" t="n">
-        <v>0.7369</v>
+        <v>1.5526</v>
       </c>
       <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>6274</t>
+          <t>6669</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>台燿</t>
+          <t>緯穎</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>230000</v>
+        <v>146000</v>
       </c>
       <c r="D44" t="n">
-        <v>0.6873</v>
+        <v>2.3959</v>
       </c>
       <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>8021</t>
+          <t>6781</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>尖點</t>
+          <t>AES-KY</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>569920</v>
+        <v>198000</v>
       </c>
       <c r="D45" t="n">
-        <v>0.6651</v>
+        <v>0.9119</v>
       </c>
       <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>3491</t>
+          <t>6805</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>昇達科</t>
+          <t>富世達</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>71000</v>
+        <v>219000</v>
       </c>
       <c r="D46" t="n">
-        <v>0.5108</v>
+        <v>1.9867</v>
       </c>
       <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2337</t>
+          <t>7751</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>旺宏</t>
+          <t>竑騰</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>671000</v>
+        <v>285000</v>
       </c>
       <c r="D47" t="n">
-        <v>0.4165</v>
+        <v>2.2836</v>
       </c>
       <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>5289</t>
+          <t>7769</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>宜鼎</t>
+          <t>鴻勁</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>90000</v>
+        <v>142000</v>
       </c>
       <c r="D48" t="n">
-        <v>0.4145</v>
+        <v>2.6207</v>
       </c>
       <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>3711</t>
+          <t>8021</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>日月光投控</t>
+          <t>尖點</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>236000</v>
+        <v>569920</v>
       </c>
       <c r="D49" t="n">
-        <v>0.41</v>
+        <v>0.6651</v>
       </c>
       <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>3324</t>
+          <t>8046</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>雙鴻</t>
+          <t>南電</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>93000</v>
+        <v>858000</v>
       </c>
       <c r="D50" t="n">
-        <v>0.4072</v>
+        <v>2.3453</v>
       </c>
       <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>3260</t>
+          <t>8299</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>威剛</t>
+          <t>群聯</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>231000</v>
+        <v>434000</v>
       </c>
       <c r="D51" t="n">
-        <v>0.4018</v>
+        <v>3.2478</v>
       </c>
       <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2344</t>
+          <t>8358</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>華邦電</t>
+          <t>金居</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>663000</v>
+        <v>1728000</v>
       </c>
       <c r="D52" t="n">
-        <v>0.2929</v>
+        <v>1.9127</v>
       </c>
       <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2449</t>
+          <t>8996</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>京元電子</t>
+          <t>高力</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>166000</v>
+        <v>715000</v>
       </c>
       <c r="D53" t="n">
-        <v>0.2069</v>
+        <v>2.9799</v>
       </c>
       <c r="E53" t="inlineStr"/>
     </row>

</xml_diff>